<commit_message>
Habille le tableau de bord aux couleurs de Multimédia Glory Guinée SARLU
Logo et nom de la société dans la page web (en-tête, pied de page, synthèse
copiée) et dans le classeur Excel (logo, en-tête d'impression, titres).
Palette accordée au bleu du logo.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Frq6RJqehZfzo9cs9xsRRC
</commit_message>
<xml_diff>
--- a/tableau-de-bord-responsable-administratif/tableau-de-bord-responsable-administratif.xlsx
+++ b/tableau-de-bord-responsable-administratif/tableau-de-bord-responsable-administratif.xlsx
@@ -26,7 +26,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="144">
+  <si>
+    <t xml:space="preserve">Multimédia Glory Guinée SARLU</t>
+  </si>
   <si>
     <t xml:space="preserve">Tableau de bord — Responsable administratif</t>
   </si>
@@ -112,7 +115,7 @@
     <t xml:space="preserve">Hypothèses : rythmes, indicateurs, cibles et marges sont des propositions à valider. Les statuts et chiffres affichés au départ sont des exemples.</t>
   </si>
   <si>
-    <t xml:space="preserve">Indicateurs de pilotage</t>
+    <t xml:space="preserve">Multimédia Glory Guinée SARLU — Indicateurs de pilotage</t>
   </si>
   <si>
     <t xml:space="preserve">Saisissez la cible et le réalisé (cellules jaunes) : l’écart et l’état se calculent seuls. Chiffres actuels : exemples.</t>
@@ -199,7 +202,7 @@
     <t xml:space="preserve">• Cibles, marges et chiffres réalisés sont des exemples proposés : remplacez-les par vos objectifs réels.</t>
   </si>
   <si>
-    <t xml:space="preserve">Missions du responsable administratif</t>
+    <t xml:space="preserve">Multimédia Glory Guinée SARLU — Missions du responsable administratif</t>
   </si>
   <si>
     <t xml:space="preserve">Choisissez le statut de la période dans la colonne H (liste déroulante). Statuts actuels : exemples.</t>
@@ -424,7 +427,7 @@
     <t xml:space="preserve">Une mission récurrente n’est jamais « terminée » : « Fait » veut dire fait pour la période en cours. À chaque nouvelle période, remettez la colonne H sur « À faire ».</t>
   </si>
   <si>
-    <t xml:space="preserve">Termes de référence — Responsable administratif</t>
+    <t xml:space="preserve">Multimédia Glory Guinée SARLU — Termes de référence — Responsable administratif</t>
   </si>
   <si>
     <t xml:space="preserve">Texte du document d’origine (orthographe corrigée). Les colonnes B et C indiquent où chaque ligne est suivie dans le classeur.</t>
@@ -470,7 +473,7 @@
     <numFmt numFmtId="169" formatCode="0"/>
     <numFmt numFmtId="170" formatCode="\+0;\-0;0"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -495,23 +498,23 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="16"/>
-      <color rgb="FF1D4F91"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF566478"/>
+      <sz val="11"/>
+      <color rgb="FF1B429D"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FF1D4F91"/>
+      <sz val="16"/>
+      <color rgb="FF1B429D"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF566478"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -566,6 +569,13 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF566478"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
@@ -598,13 +608,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE4EDF9"/>
-        <bgColor rgb="FFEEF1F5"/>
+        <fgColor rgb="FFE3E9F7"/>
+        <bgColor rgb="FFDCE2EB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1D4F91"/>
+        <fgColor rgb="FF1B429D"/>
         <bgColor rgb="FF003366"/>
       </patternFill>
     </fill>
@@ -694,7 +704,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -707,7 +717,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -775,11 +789,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -791,11 +809,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="16" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -807,11 +825,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="16" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -819,7 +837,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -827,7 +845,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -903,7 +921,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF1D4F91"/>
+          <fgColor rgb="FF1B429D"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -934,7 +952,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFE4EDF9"/>
+          <fgColor rgb="FFE3E9F7"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -985,11 +1003,11 @@
         <charset val="1"/>
         <family val="0"/>
         <b val="1"/>
-        <color rgb="FF1D4F91"/>
+        <color rgb="FF1B429D"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFE4EDF9"/>
+          <bgColor rgb="FFE3E9F7"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1043,7 +1061,7 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFE4EDF9"/>
+      <rgbColor rgb="FFE3E9F7"/>
       <rgbColor rgb="FFEEF1F5"/>
       <rgbColor rgb="FFFDF0D5"/>
       <rgbColor rgb="FFDCE2EB"/>
@@ -1064,7 +1082,7 @@
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FFB3261E"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF1D4F91"/>
+      <rgbColor rgb="FF1B429D"/>
       <rgbColor rgb="FF333333"/>
     </indexedColors>
   </colors>
@@ -1236,11 +1254,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="1d4f91"/>
+              <a:srgbClr val="1b429d"/>
             </a:solidFill>
             <a:ln w="0">
               <a:solidFill>
-                <a:srgbClr val="1d4f91"/>
+                <a:srgbClr val="1b429d"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
@@ -1534,11 +1552,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="33478551"/>
-        <c:axId val="33514319"/>
+        <c:axId val="83873311"/>
+        <c:axId val="29672029"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="33478551"/>
+        <c:axId val="83873311"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1570,7 +1588,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="33514319"/>
+        <c:crossAx val="29672029"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1578,7 +1596,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="33514319"/>
+        <c:axId val="29672029"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1610,7 +1628,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="33478551"/>
+        <c:crossAx val="83873311"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1936,11 +1954,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="86056954"/>
-        <c:axId val="68199084"/>
+        <c:axId val="65983716"/>
+        <c:axId val="35577680"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="86056954"/>
+        <c:axId val="65983716"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1972,7 +1990,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="68199084"/>
+        <c:crossAx val="35577680"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1980,7 +1998,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="68199084"/>
+        <c:axId val="35577680"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2012,7 +2030,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86056954"/>
+        <c:crossAx val="65983716"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2061,7 +2079,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="0" y="5067360"/>
+        <a:off x="0" y="5172120"/>
         <a:ext cx="5399640" cy="3059640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -2091,7 +2109,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="5356800" y="5067360"/>
+        <a:off x="5356800" y="5172120"/>
         <a:ext cx="4319640" cy="3059640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -2100,6 +2118,43 @@
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>742680</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>161640</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 3" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8317080" y="0"/>
+          <a:ext cx="742680" cy="742680"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -2287,7 +2342,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF1D4F91"/>
+    <tabColor rgb="FF1B429D"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:I40"/>
@@ -2298,433 +2353,438 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
+    <row r="3" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
+      <c r="A4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5"/>
-      <c r="B5" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="7" t="s">
+      <c r="A5" s="6"/>
+      <c r="B5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="C5" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="D5" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="E5" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="F5" s="6" t="s">
         <v>8</v>
       </c>
+      <c r="G5" s="6" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="11" t="n">
+      <c r="A6" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="12" t="n">
         <f aca="false">COUNTIF(Indicateurs!$H$6:$H$16,B$5)</f>
         <v>5</v>
       </c>
-      <c r="C6" s="11" t="n">
+      <c r="C6" s="12" t="n">
         <f aca="false">COUNTIF(Indicateurs!$H$6:$H$16,C$5)</f>
         <v>4</v>
       </c>
-      <c r="D6" s="11" t="n">
+      <c r="D6" s="12" t="n">
         <f aca="false">COUNTIF(Indicateurs!$H$6:$H$16,D$5)</f>
         <v>2</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="12" t="n">
         <f aca="false">COUNTIF(Indicateurs!$H$6:$H$16,E$5)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="F6" s="12" t="n">
         <f aca="false">SUM(B6:E6)</f>
         <v>11</v>
       </c>
-      <c r="G6" s="12" t="n">
+      <c r="G6" s="13" t="n">
         <f aca="false">IF(F6=0,0,B6/F6)</f>
         <v>0.454545454545455</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5"/>
-      <c r="B7" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="5" t="s">
+      <c r="A7" s="6"/>
+      <c r="B7" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="C7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="D7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G7" s="5" t="s">
+      <c r="E7" s="10" t="s">
         <v>14</v>
       </c>
+      <c r="F7" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="11" t="n">
+      <c r="A8" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="12" t="n">
         <f aca="false">COUNTIF(Missions!$H$5:$H$21,B$7)</f>
         <v>8</v>
       </c>
-      <c r="C8" s="11" t="n">
+      <c r="C8" s="12" t="n">
         <f aca="false">COUNTIF(Missions!$H$5:$H$21,C$7)</f>
         <v>4</v>
       </c>
-      <c r="D8" s="11" t="n">
+      <c r="D8" s="12" t="n">
         <f aca="false">COUNTIF(Missions!$H$5:$H$21,D$7)</f>
         <v>2</v>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="12" t="n">
         <f aca="false">COUNTIF(Missions!$H$5:$H$21,E$7)</f>
         <v>3</v>
       </c>
-      <c r="F8" s="11" t="n">
+      <c r="F8" s="12" t="n">
         <f aca="false">SUM(B8:E8)</f>
         <v>17</v>
       </c>
-      <c r="G8" s="12" t="n">
+      <c r="G8" s="13" t="n">
         <f aca="false">IF(F8=0,0,B8/F8)</f>
         <v>0.470588235294118</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
+      <c r="A10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="5" t="s">
+      <c r="A11" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="5" t="s">
+      <c r="B11" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="E11" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="F11" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="H11" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="I11" s="5" t="s">
+      <c r="G11" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H11" s="6" t="s">
         <v>20</v>
       </c>
+      <c r="I11" s="6" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="14" t="n">
+      <c r="A12" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="15" t="n">
         <f aca="false">COUNTIF(Missions!$B$5:$B$21,$A12)</f>
         <v>2</v>
       </c>
-      <c r="C12" s="14" t="n">
+      <c r="C12" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A12,Missions!$H$5:$H$21,C$11)</f>
         <v>2</v>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A12,Missions!$H$5:$H$21,D$11)</f>
         <v>0</v>
       </c>
-      <c r="E12" s="14" t="n">
+      <c r="E12" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A12,Missions!$H$5:$H$21,E$11)</f>
         <v>0</v>
       </c>
-      <c r="F12" s="14" t="n">
+      <c r="F12" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A12,Missions!$H$5:$H$21,F$11)</f>
         <v>0</v>
       </c>
-      <c r="G12" s="15" t="n">
+      <c r="G12" s="16" t="n">
         <f aca="false">IF($B12=0,0,C12/$B12)</f>
         <v>1</v>
       </c>
-      <c r="H12" s="14" t="n">
+      <c r="H12" s="15" t="n">
         <f aca="false">COUNTIFS(Indicateurs!$A$6:$A$16,$A12,Indicateurs!$H$6:$H$16,"Hors cible")</f>
         <v>0</v>
       </c>
-      <c r="I12" s="14" t="n">
+      <c r="I12" s="15" t="n">
         <f aca="false">COUNTIFS(Indicateurs!$A$6:$A$16,$A12,Indicateurs!$H$6:$H$16,"À surveiller")</f>
         <v>2</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="14" t="n">
+      <c r="A13" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="15" t="n">
         <f aca="false">COUNTIF(Missions!$B$5:$B$21,$A13)</f>
         <v>3</v>
       </c>
-      <c r="C13" s="14" t="n">
+      <c r="C13" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A13,Missions!$H$5:$H$21,C$11)</f>
         <v>2</v>
       </c>
-      <c r="D13" s="14" t="n">
+      <c r="D13" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A13,Missions!$H$5:$H$21,D$11)</f>
         <v>1</v>
       </c>
-      <c r="E13" s="14" t="n">
+      <c r="E13" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A13,Missions!$H$5:$H$21,E$11)</f>
         <v>0</v>
       </c>
-      <c r="F13" s="14" t="n">
+      <c r="F13" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A13,Missions!$H$5:$H$21,F$11)</f>
         <v>0</v>
       </c>
-      <c r="G13" s="15" t="n">
+      <c r="G13" s="16" t="n">
         <f aca="false">IF($B13=0,0,C13/$B13)</f>
         <v>0.666666666666667</v>
       </c>
-      <c r="H13" s="14" t="n">
+      <c r="H13" s="15" t="n">
         <f aca="false">COUNTIFS(Indicateurs!$A$6:$A$16,$A13,Indicateurs!$H$6:$H$16,"Hors cible")</f>
         <v>1</v>
       </c>
-      <c r="I13" s="14" t="n">
+      <c r="I13" s="15" t="n">
         <f aca="false">COUNTIFS(Indicateurs!$A$6:$A$16,$A13,Indicateurs!$H$6:$H$16,"À surveiller")</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="B14" s="14" t="n">
+      <c r="A14" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="15" t="n">
         <f aca="false">COUNTIF(Missions!$B$5:$B$21,$A14)</f>
         <v>3</v>
       </c>
-      <c r="C14" s="14" t="n">
+      <c r="C14" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A14,Missions!$H$5:$H$21,C$11)</f>
         <v>1</v>
       </c>
-      <c r="D14" s="14" t="n">
+      <c r="D14" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A14,Missions!$H$5:$H$21,D$11)</f>
         <v>1</v>
       </c>
-      <c r="E14" s="14" t="n">
+      <c r="E14" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A14,Missions!$H$5:$H$21,E$11)</f>
         <v>1</v>
       </c>
-      <c r="F14" s="14" t="n">
+      <c r="F14" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A14,Missions!$H$5:$H$21,F$11)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="15" t="n">
+      <c r="G14" s="16" t="n">
         <f aca="false">IF($B14=0,0,C14/$B14)</f>
         <v>0.333333333333333</v>
       </c>
-      <c r="H14" s="14" t="n">
+      <c r="H14" s="15" t="n">
         <f aca="false">COUNTIFS(Indicateurs!$A$6:$A$16,$A14,Indicateurs!$H$6:$H$16,"Hors cible")</f>
         <v>0</v>
       </c>
-      <c r="I14" s="14" t="n">
+      <c r="I14" s="15" t="n">
         <f aca="false">COUNTIFS(Indicateurs!$A$6:$A$16,$A14,Indicateurs!$H$6:$H$16,"À surveiller")</f>
         <v>1</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B15" s="14" t="n">
+      <c r="A15" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="15" t="n">
         <f aca="false">COUNTIF(Missions!$B$5:$B$21,$A15)</f>
         <v>5</v>
       </c>
-      <c r="C15" s="14" t="n">
+      <c r="C15" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A15,Missions!$H$5:$H$21,C$11)</f>
         <v>1</v>
       </c>
-      <c r="D15" s="14" t="n">
+      <c r="D15" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A15,Missions!$H$5:$H$21,D$11)</f>
         <v>1</v>
       </c>
-      <c r="E15" s="14" t="n">
+      <c r="E15" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A15,Missions!$H$5:$H$21,E$11)</f>
         <v>1</v>
       </c>
-      <c r="F15" s="14" t="n">
+      <c r="F15" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A15,Missions!$H$5:$H$21,F$11)</f>
         <v>2</v>
       </c>
-      <c r="G15" s="15" t="n">
+      <c r="G15" s="16" t="n">
         <f aca="false">IF($B15=0,0,C15/$B15)</f>
         <v>0.2</v>
       </c>
-      <c r="H15" s="14" t="n">
+      <c r="H15" s="15" t="n">
         <f aca="false">COUNTIFS(Indicateurs!$A$6:$A$16,$A15,Indicateurs!$H$6:$H$16,"Hors cible")</f>
         <v>1</v>
       </c>
-      <c r="I15" s="14" t="n">
+      <c r="I15" s="15" t="n">
         <f aca="false">COUNTIFS(Indicateurs!$A$6:$A$16,$A15,Indicateurs!$H$6:$H$16,"À surveiller")</f>
         <v>1</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="B16" s="14" t="n">
+      <c r="A16" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="15" t="n">
         <f aca="false">COUNTIF(Missions!$B$5:$B$21,$A16)</f>
         <v>3</v>
       </c>
-      <c r="C16" s="14" t="n">
+      <c r="C16" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A16,Missions!$H$5:$H$21,C$11)</f>
         <v>2</v>
       </c>
-      <c r="D16" s="14" t="n">
+      <c r="D16" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A16,Missions!$H$5:$H$21,D$11)</f>
         <v>0</v>
       </c>
-      <c r="E16" s="14" t="n">
+      <c r="E16" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A16,Missions!$H$5:$H$21,E$11)</f>
         <v>0</v>
       </c>
-      <c r="F16" s="14" t="n">
+      <c r="F16" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A16,Missions!$H$5:$H$21,F$11)</f>
         <v>1</v>
       </c>
-      <c r="G16" s="15" t="n">
+      <c r="G16" s="16" t="n">
         <f aca="false">IF($B16=0,0,C16/$B16)</f>
         <v>0.666666666666667</v>
       </c>
-      <c r="H16" s="14" t="n">
+      <c r="H16" s="15" t="n">
         <f aca="false">COUNTIFS(Indicateurs!$A$6:$A$16,$A16,Indicateurs!$H$6:$H$16,"Hors cible")</f>
         <v>0</v>
       </c>
-      <c r="I16" s="14" t="n">
+      <c r="I16" s="15" t="n">
         <f aca="false">COUNTIFS(Indicateurs!$A$6:$A$16,$A16,Indicateurs!$H$6:$H$16,"À surveiller")</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="B17" s="14" t="n">
+      <c r="A17" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="15" t="n">
         <f aca="false">COUNTIF(Missions!$B$5:$B$21,$A17)</f>
         <v>1</v>
       </c>
-      <c r="C17" s="14" t="n">
+      <c r="C17" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A17,Missions!$H$5:$H$21,C$11)</f>
         <v>0</v>
       </c>
-      <c r="D17" s="14" t="n">
+      <c r="D17" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A17,Missions!$H$5:$H$21,D$11)</f>
         <v>1</v>
       </c>
-      <c r="E17" s="14" t="n">
+      <c r="E17" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A17,Missions!$H$5:$H$21,E$11)</f>
         <v>0</v>
       </c>
-      <c r="F17" s="14" t="n">
+      <c r="F17" s="15" t="n">
         <f aca="false">COUNTIFS(Missions!$B$5:$B$21,$A17,Missions!$H$5:$H$21,F$11)</f>
         <v>0</v>
       </c>
-      <c r="G17" s="15" t="n">
+      <c r="G17" s="16" t="n">
         <f aca="false">IF($B17=0,0,C17/$B17)</f>
         <v>0</v>
       </c>
-      <c r="H17" s="14" t="n">
+      <c r="H17" s="15" t="n">
         <f aca="false">COUNTIFS(Indicateurs!$A$6:$A$16,$A17,Indicateurs!$H$6:$H$16,"Hors cible")</f>
         <v>0</v>
       </c>
-      <c r="I17" s="14" t="n">
+      <c r="I17" s="15" t="n">
         <f aca="false">COUNTIFS(Indicateurs!$A$6:$A$16,$A17,Indicateurs!$H$6:$H$16,"À surveiller")</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="B18" s="17" t="n">
+      <c r="A18" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18" s="18" t="n">
         <f aca="false">SUM(B12:B17)</f>
         <v>17</v>
       </c>
-      <c r="C18" s="17" t="n">
+      <c r="C18" s="18" t="n">
         <f aca="false">SUM(C12:C17)</f>
         <v>8</v>
       </c>
-      <c r="D18" s="17" t="n">
+      <c r="D18" s="18" t="n">
         <f aca="false">SUM(D12:D17)</f>
         <v>4</v>
       </c>
-      <c r="E18" s="17" t="n">
+      <c r="E18" s="18" t="n">
         <f aca="false">SUM(E12:E17)</f>
         <v>2</v>
       </c>
-      <c r="F18" s="17" t="n">
+      <c r="F18" s="18" t="n">
         <f aca="false">SUM(F12:F17)</f>
         <v>3</v>
       </c>
-      <c r="G18" s="18" t="n">
+      <c r="G18" s="19" t="n">
         <f aca="false">IF(B18=0,0,C18/B18)</f>
         <v>0.470588235294118</v>
       </c>
-      <c r="H18" s="17" t="n">
+      <c r="H18" s="18" t="n">
         <f aca="false">SUM(H12:H17)</f>
         <v>2</v>
       </c>
-      <c r="I18" s="17" t="n">
+      <c r="I18" s="18" t="n">
         <f aca="false">SUM(I12:I17)</f>
         <v>4</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="19" t="s">
-        <v>27</v>
+      <c r="A40" s="20" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -2744,11 +2804,11 @@
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
+    <oddHeader>&amp;C&amp;10 Multimédia Glory Guinée SARLU</oddHeader>
+    <oddFooter>&amp;C&amp;9 Page &amp;P sur &amp;N</oddFooter>
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -2772,371 +2832,371 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>28</v>
+      <c r="A1" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>29</v>
+      <c r="A2" s="21" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" s="21" t="n">
+      <c r="A3" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="23" t="n">
         <v>0.9</v>
       </c>
-      <c r="D3" s="19" t="s">
-        <v>31</v>
+      <c r="D3" s="20" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" s="5" t="s">
+      <c r="A5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="F5" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="G5" s="6" t="s">
         <v>38</v>
       </c>
+      <c r="H5" s="6" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="C6" s="23" t="s">
+      <c r="A6" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="D6" s="24"/>
-      <c r="E6" s="25" t="n">
+      <c r="C6" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" s="26"/>
+      <c r="E6" s="27" t="n">
         <v>0.95</v>
       </c>
-      <c r="F6" s="25" t="n">
+      <c r="F6" s="27" t="n">
         <v>0.92</v>
       </c>
-      <c r="G6" s="26" t="n">
+      <c r="G6" s="28" t="n">
         <f aca="false">IF(OR(E6="",F6=""),"",F6-E6)</f>
         <v>-0.0299999999999999</v>
       </c>
-      <c r="H6" s="27" t="str">
+      <c r="H6" s="29" t="str">
         <f aca="false">IF(OR(E6="",F6=""),"À renseigner",IF(C6="≥",IF(F6&gt;=E6,"Atteint",IF(F6&gt;=E6*$C$3,"À surveiller","Hors cible")),IF(F6&lt;=E6,"Atteint",IF(F6&lt;=E6+D6,"À surveiller","Hors cible"))))</f>
         <v>À surveiller</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" s="23" t="s">
+      <c r="A7" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="24" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="28" t="n">
+      <c r="C7" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="30" t="n">
         <v>3</v>
       </c>
-      <c r="E7" s="29" t="n">
+      <c r="E7" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="F7" s="29" t="n">
+      <c r="F7" s="31" t="n">
         <v>4</v>
       </c>
-      <c r="G7" s="30" t="n">
+      <c r="G7" s="32" t="n">
         <f aca="false">IF(OR(E7="",F7=""),"",F7-E7)</f>
         <v>2</v>
       </c>
-      <c r="H7" s="27" t="str">
+      <c r="H7" s="29" t="str">
         <f aca="false">IF(OR(E7="",F7=""),"À renseigner",IF(C7="≥",IF(F7&gt;=E7,"Atteint",IF(F7&gt;=E7*$C$3,"À surveiller","Hors cible")),IF(F7&lt;=E7,"Atteint",IF(F7&lt;=E7+D7,"À surveiller","Hors cible"))))</f>
         <v>À surveiller</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" s="22" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8" s="24"/>
-      <c r="E8" s="25" t="n">
+      <c r="A8" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="26"/>
+      <c r="E8" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="25" t="n">
+      <c r="F8" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="26" t="n">
+      <c r="G8" s="28" t="n">
         <f aca="false">IF(OR(E8="",F8=""),"",F8-E8)</f>
         <v>0</v>
       </c>
-      <c r="H8" s="27" t="str">
+      <c r="H8" s="29" t="str">
         <f aca="false">IF(OR(E8="",F8=""),"À renseigner",IF(C8="≥",IF(F8&gt;=E8,"Atteint",IF(F8&gt;=E8*$C$3,"À surveiller","Hors cible")),IF(F8&lt;=E8,"Atteint",IF(F8&lt;=E8+D8,"À surveiller","Hors cible"))))</f>
         <v>Atteint</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="22" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="D9" s="28" t="n">
+      <c r="A9" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="24" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="D9" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="29" t="n">
+      <c r="E9" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="29" t="n">
+      <c r="F9" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="G9" s="30" t="n">
+      <c r="G9" s="32" t="n">
         <f aca="false">IF(OR(E9="",F9=""),"",F9-E9)</f>
         <v>2</v>
       </c>
-      <c r="H9" s="27" t="str">
+      <c r="H9" s="29" t="str">
         <f aca="false">IF(OR(E9="",F9=""),"À renseigner",IF(C9="≥",IF(F9&gt;=E9,"Atteint",IF(F9&gt;=E9*$C$3,"À surveiller","Hors cible")),IF(F9&lt;=E9,"Atteint",IF(F9&lt;=E9+D9,"À surveiller","Hors cible"))))</f>
         <v>Hors cible</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="22" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="D10" s="24"/>
-      <c r="E10" s="25" t="n">
+      <c r="A10" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="26"/>
+      <c r="E10" s="27" t="n">
         <v>0.98</v>
       </c>
-      <c r="F10" s="25" t="n">
+      <c r="F10" s="27" t="n">
         <v>0.96</v>
       </c>
-      <c r="G10" s="26" t="n">
+      <c r="G10" s="28" t="n">
         <f aca="false">IF(OR(E10="",F10=""),"",F10-E10)</f>
         <v>-0.02</v>
       </c>
-      <c r="H10" s="27" t="str">
+      <c r="H10" s="29" t="str">
         <f aca="false">IF(OR(E10="",F10=""),"À renseigner",IF(C10="≥",IF(F10&gt;=E10,"Atteint",IF(F10&gt;=E10*$C$3,"À surveiller","Hors cible")),IF(F10&lt;=E10,"Atteint",IF(F10&lt;=E10+D10,"À surveiller","Hors cible"))))</f>
         <v>À surveiller</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="22" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="D11" s="28" t="n">
+      <c r="A11" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="29" t="n">
+      <c r="E11" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="29" t="n">
+      <c r="F11" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="30" t="n">
+      <c r="G11" s="32" t="n">
         <f aca="false">IF(OR(E11="",F11=""),"",F11-E11)</f>
         <v>0</v>
       </c>
-      <c r="H11" s="27" t="str">
+      <c r="H11" s="29" t="str">
         <f aca="false">IF(OR(E11="",F11=""),"À renseigner",IF(C11="≥",IF(F11&gt;=E11,"Atteint",IF(F11&gt;=E11*$C$3,"À surveiller","Hors cible")),IF(F11&lt;=E11,"Atteint",IF(F11&lt;=E11+D11,"À surveiller","Hors cible"))))</f>
         <v>Atteint</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="22" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" s="22" t="s">
-        <v>47</v>
-      </c>
-      <c r="C12" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12" s="28" t="n">
+      <c r="A12" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="29" t="n">
+      <c r="E12" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="29" t="n">
+      <c r="F12" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="30" t="n">
+      <c r="G12" s="32" t="n">
         <f aca="false">IF(OR(E12="",F12=""),"",F12-E12)</f>
         <v>0</v>
       </c>
-      <c r="H12" s="27" t="str">
+      <c r="H12" s="29" t="str">
         <f aca="false">IF(OR(E12="",F12=""),"À renseigner",IF(C12="≥",IF(F12&gt;=E12,"Atteint",IF(F12&gt;=E12*$C$3,"À surveiller","Hors cible")),IF(F12&lt;=E12,"Atteint",IF(F12&lt;=E12+D12,"À surveiller","Hors cible"))))</f>
         <v>Atteint</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="22" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" s="22" t="s">
-        <v>48</v>
-      </c>
-      <c r="C13" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="D13" s="24"/>
-      <c r="E13" s="25" t="n">
+      <c r="A13" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="26"/>
+      <c r="E13" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="25" t="n">
+      <c r="F13" s="27" t="n">
         <v>0.97</v>
       </c>
-      <c r="G13" s="26" t="n">
+      <c r="G13" s="28" t="n">
         <f aca="false">IF(OR(E13="",F13=""),"",F13-E13)</f>
         <v>-0.03</v>
       </c>
-      <c r="H13" s="27" t="str">
+      <c r="H13" s="29" t="str">
         <f aca="false">IF(OR(E13="",F13=""),"À renseigner",IF(C13="≥",IF(F13&gt;=E13,"Atteint",IF(F13&gt;=E13*$C$3,"À surveiller","Hors cible")),IF(F13&lt;=E13,"Atteint",IF(F13&lt;=E13+D13,"À surveiller","Hors cible"))))</f>
         <v>À surveiller</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="22" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" s="22" t="s">
-        <v>49</v>
-      </c>
-      <c r="C14" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" s="28" t="n">
+      <c r="A14" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" s="25" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="29" t="n">
+      <c r="E14" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="29" t="n">
+      <c r="F14" s="31" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="30" t="n">
+      <c r="G14" s="32" t="n">
         <f aca="false">IF(OR(E14="",F14=""),"",F14-E14)</f>
         <v>3</v>
       </c>
-      <c r="H14" s="27" t="str">
+      <c r="H14" s="29" t="str">
         <f aca="false">IF(OR(E14="",F14=""),"À renseigner",IF(C14="≥",IF(F14&gt;=E14,"Atteint",IF(F14&gt;=E14*$C$3,"À surveiller","Hors cible")),IF(F14&lt;=E14,"Atteint",IF(F14&lt;=E14+D14,"À surveiller","Hors cible"))))</f>
         <v>Hors cible</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B15" s="22" t="s">
-        <v>50</v>
-      </c>
-      <c r="C15" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="D15" s="24"/>
-      <c r="E15" s="25" t="n">
+      <c r="A15" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" s="26"/>
+      <c r="E15" s="27" t="n">
         <v>0.9</v>
       </c>
-      <c r="F15" s="25" t="n">
+      <c r="F15" s="27" t="n">
         <v>0.9</v>
       </c>
-      <c r="G15" s="26" t="n">
+      <c r="G15" s="28" t="n">
         <f aca="false">IF(OR(E15="",F15=""),"",F15-E15)</f>
         <v>0</v>
       </c>
-      <c r="H15" s="27" t="str">
+      <c r="H15" s="29" t="str">
         <f aca="false">IF(OR(E15="",F15=""),"À renseigner",IF(C15="≥",IF(F15&gt;=E15,"Atteint",IF(F15&gt;=E15*$C$3,"À surveiller","Hors cible")),IF(F15&lt;=E15,"Atteint",IF(F15&lt;=E15+D15,"À surveiller","Hors cible"))))</f>
         <v>Atteint</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="B16" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="C16" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="D16" s="24"/>
-      <c r="E16" s="25" t="n">
+      <c r="A16" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" s="26"/>
+      <c r="E16" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="F16" s="25" t="n">
+      <c r="F16" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="G16" s="26" t="n">
+      <c r="G16" s="28" t="n">
         <f aca="false">IF(OR(E16="",F16=""),"",F16-E16)</f>
         <v>0</v>
       </c>
-      <c r="H16" s="27" t="str">
+      <c r="H16" s="29" t="str">
         <f aca="false">IF(OR(E16="",F16=""),"À renseigner",IF(C16="≥",IF(F16&gt;=E16,"Atteint",IF(F16&gt;=E16*$C$3,"À surveiller","Hors cible")),IF(F16&lt;=E16,"Atteint",IF(F16&lt;=E16+D16,"À surveiller","Hors cible"))))</f>
         <v>Atteint</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="31" t="s">
-        <v>52</v>
+      <c r="A18" s="33" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
-        <v>53</v>
+      <c r="A19" s="20" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="19" t="s">
-        <v>54</v>
+      <c r="A20" s="20" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="19" t="s">
-        <v>55</v>
+      <c r="A21" s="20" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="19" t="s">
-        <v>56</v>
+      <c r="A22" s="20" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -3152,11 +3212,11 @@
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
+    <oddHeader>&amp;C&amp;10 Multimédia Glory Guinée SARLU</oddHeader>
+    <oddFooter>&amp;C&amp;9 Page &amp;P sur &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -3179,465 +3239,465 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>57</v>
+      <c r="A1" s="2" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>58</v>
+      <c r="A2" s="21" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
-        <v>59</v>
+      <c r="A3" s="20" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="B4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="F4" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="G4" s="6" t="s">
         <v>66</v>
       </c>
+      <c r="H4" s="6" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="B5" s="32" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="32" t="s">
+      <c r="A5" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32" t="s">
+      <c r="B5" s="34" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="F5" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="G5" s="32" t="s">
+      <c r="D5" s="34"/>
+      <c r="E5" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="H5" s="33" t="s">
-        <v>10</v>
+      <c r="F5" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="G5" s="34" t="s">
+        <v>71</v>
+      </c>
+      <c r="H5" s="35" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="32" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" s="32" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="32" t="s">
+      <c r="A6" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="D6" s="32" t="s">
+      <c r="B6" s="34" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="E6" s="32" t="s">
+      <c r="D6" s="34" t="s">
         <v>74</v>
       </c>
-      <c r="F6" s="32" t="s">
-        <v>74</v>
-      </c>
-      <c r="G6" s="32" t="s">
+      <c r="E6" s="34" t="s">
         <v>75</v>
       </c>
-      <c r="H6" s="33" t="s">
-        <v>10</v>
+      <c r="F6" s="34" t="s">
+        <v>75</v>
+      </c>
+      <c r="G6" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="H6" s="35" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="32" t="s">
-        <v>76</v>
-      </c>
-      <c r="B7" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" s="32" t="s">
+      <c r="A7" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="F7" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="G7" s="32" t="s">
+      <c r="B7" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="34" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="33" t="s">
-        <v>10</v>
+      <c r="D7" s="34"/>
+      <c r="E7" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="F7" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="G7" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="H7" s="35" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="32" t="s">
-        <v>79</v>
-      </c>
-      <c r="B8" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" s="32" t="s">
+      <c r="A8" s="34" t="s">
         <v>80</v>
       </c>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32" t="s">
+      <c r="B8" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="34" t="s">
         <v>81</v>
       </c>
-      <c r="F8" s="32" t="s">
+      <c r="D8" s="34"/>
+      <c r="E8" s="34" t="s">
         <v>82</v>
       </c>
-      <c r="G8" s="32" t="s">
+      <c r="F8" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="H8" s="33" t="s">
-        <v>10</v>
+      <c r="G8" s="34" t="s">
+        <v>84</v>
+      </c>
+      <c r="H8" s="35" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="32" t="s">
-        <v>84</v>
-      </c>
-      <c r="B9" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="C9" s="32" t="s">
+      <c r="A9" s="34" t="s">
         <v>85</v>
       </c>
-      <c r="D9" s="32"/>
-      <c r="E9" s="32" t="s">
+      <c r="B9" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="34" t="s">
         <v>86</v>
       </c>
-      <c r="F9" s="32" t="s">
-        <v>82</v>
-      </c>
-      <c r="G9" s="32" t="s">
+      <c r="D9" s="34"/>
+      <c r="E9" s="34" t="s">
         <v>87</v>
       </c>
-      <c r="H9" s="33" t="s">
+      <c r="F9" s="34" t="s">
+        <v>83</v>
+      </c>
+      <c r="G9" s="34" t="s">
+        <v>88</v>
+      </c>
+      <c r="H9" s="35" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="34" t="s">
+        <v>89</v>
+      </c>
+      <c r="B10" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="34" t="s">
+        <v>90</v>
+      </c>
+      <c r="D10" s="34"/>
+      <c r="E10" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="F10" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="G10" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="H10" s="35" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="32" t="s">
-        <v>88</v>
-      </c>
-      <c r="B10" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" s="32" t="s">
-        <v>89</v>
-      </c>
-      <c r="D10" s="32"/>
-      <c r="E10" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="F10" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="G10" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="H10" s="33" t="s">
-        <v>10</v>
-      </c>
-    </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="32" t="s">
-        <v>91</v>
-      </c>
-      <c r="B11" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="32" t="s">
+      <c r="A11" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="D11" s="32" t="s">
+      <c r="B11" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="34" t="s">
         <v>93</v>
       </c>
-      <c r="E11" s="32" t="s">
+      <c r="D11" s="34" t="s">
         <v>94</v>
       </c>
-      <c r="F11" s="32" t="s">
-        <v>94</v>
-      </c>
-      <c r="G11" s="32" t="s">
+      <c r="E11" s="34" t="s">
         <v>95</v>
       </c>
-      <c r="H11" s="33" t="s">
+      <c r="F11" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="G11" s="34" t="s">
+        <v>96</v>
+      </c>
+      <c r="H11" s="35" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="34" t="s">
+        <v>97</v>
+      </c>
+      <c r="B12" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="34" t="s">
+        <v>98</v>
+      </c>
+      <c r="D12" s="34"/>
+      <c r="E12" s="34" t="s">
+        <v>99</v>
+      </c>
+      <c r="F12" s="34" t="s">
+        <v>83</v>
+      </c>
+      <c r="G12" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="H12" s="35" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="34" t="s">
+        <v>101</v>
+      </c>
+      <c r="B13" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="34" t="s">
+        <v>102</v>
+      </c>
+      <c r="D13" s="34"/>
+      <c r="E13" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="F13" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="G13" s="34" t="s">
+        <v>104</v>
+      </c>
+      <c r="H13" s="35" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="B12" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="32" t="s">
-        <v>97</v>
-      </c>
-      <c r="D12" s="32"/>
-      <c r="E12" s="32" t="s">
-        <v>98</v>
-      </c>
-      <c r="F12" s="32" t="s">
-        <v>82</v>
-      </c>
-      <c r="G12" s="32" t="s">
-        <v>99</v>
-      </c>
-      <c r="H12" s="33" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="34" t="s">
+        <v>105</v>
+      </c>
+      <c r="B14" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="34" t="s">
+        <v>106</v>
+      </c>
+      <c r="D14" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="E14" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="F14" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="G14" s="34" t="s">
+        <v>108</v>
+      </c>
+      <c r="H14" s="35" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="32" t="s">
-        <v>100</v>
-      </c>
-      <c r="B13" s="32" t="s">
-        <v>24</v>
-      </c>
-      <c r="C13" s="32" t="s">
-        <v>101</v>
-      </c>
-      <c r="D13" s="32"/>
-      <c r="E13" s="32" t="s">
-        <v>102</v>
-      </c>
-      <c r="F13" s="32" t="s">
-        <v>102</v>
-      </c>
-      <c r="G13" s="32" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="34" t="s">
+        <v>109</v>
+      </c>
+      <c r="B15" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="34" t="s">
+        <v>110</v>
+      </c>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34" t="s">
         <v>103</v>
       </c>
-      <c r="H13" s="33" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="32" t="s">
-        <v>104</v>
-      </c>
-      <c r="B14" s="32" t="s">
-        <v>24</v>
-      </c>
-      <c r="C14" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="D14" s="32" t="s">
-        <v>106</v>
-      </c>
-      <c r="E14" s="32" t="s">
-        <v>94</v>
-      </c>
-      <c r="F14" s="32" t="s">
-        <v>94</v>
-      </c>
-      <c r="G14" s="32" t="s">
-        <v>107</v>
-      </c>
-      <c r="H14" s="33" t="s">
+      <c r="F15" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="G15" s="34" t="s">
+        <v>111</v>
+      </c>
+      <c r="H15" s="35" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="34" t="s">
+        <v>112</v>
+      </c>
+      <c r="B16" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="34" t="s">
+        <v>113</v>
+      </c>
+      <c r="D16" s="34" t="s">
+        <v>114</v>
+      </c>
+      <c r="E16" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="F16" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="G16" s="34" t="s">
+        <v>115</v>
+      </c>
+      <c r="H16" s="35" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="34" t="s">
+        <v>116</v>
+      </c>
+      <c r="B17" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="34" t="s">
+        <v>117</v>
+      </c>
+      <c r="D17" s="34"/>
+      <c r="E17" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="F17" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="G17" s="34" t="s">
+        <v>118</v>
+      </c>
+      <c r="H17" s="35" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="34" t="s">
+        <v>119</v>
+      </c>
+      <c r="B18" s="34" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="34" t="s">
+        <v>120</v>
+      </c>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="F18" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="G18" s="34" t="s">
+        <v>121</v>
+      </c>
+      <c r="H18" s="35" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="32" t="s">
-        <v>108</v>
-      </c>
-      <c r="B15" s="32" t="s">
-        <v>24</v>
-      </c>
-      <c r="C15" s="32" t="s">
-        <v>109</v>
-      </c>
-      <c r="D15" s="32"/>
-      <c r="E15" s="32" t="s">
-        <v>102</v>
-      </c>
-      <c r="F15" s="32" t="s">
-        <v>102</v>
-      </c>
-      <c r="G15" s="32" t="s">
-        <v>110</v>
-      </c>
-      <c r="H15" s="33" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="32" t="s">
-        <v>111</v>
-      </c>
-      <c r="B16" s="32" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16" s="32" t="s">
-        <v>112</v>
-      </c>
-      <c r="D16" s="32" t="s">
-        <v>113</v>
-      </c>
-      <c r="E16" s="32" t="s">
-        <v>94</v>
-      </c>
-      <c r="F16" s="32" t="s">
-        <v>94</v>
-      </c>
-      <c r="G16" s="32" t="s">
-        <v>114</v>
-      </c>
-      <c r="H16" s="33" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="32" t="s">
-        <v>115</v>
-      </c>
-      <c r="B17" s="32" t="s">
-        <v>24</v>
-      </c>
-      <c r="C17" s="32" t="s">
-        <v>116</v>
-      </c>
-      <c r="D17" s="32"/>
-      <c r="E17" s="32" t="s">
-        <v>102</v>
-      </c>
-      <c r="F17" s="32" t="s">
-        <v>102</v>
-      </c>
-      <c r="G17" s="32" t="s">
-        <v>117</v>
-      </c>
-      <c r="H17" s="33" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="B19" s="34" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="34" t="s">
+        <v>123</v>
+      </c>
+      <c r="D19" s="34"/>
+      <c r="E19" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="F19" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="G19" s="34" t="s">
+        <v>124</v>
+      </c>
+      <c r="H19" s="35" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="34" t="s">
+        <v>125</v>
+      </c>
+      <c r="B20" s="34" t="s">
+        <v>26</v>
+      </c>
+      <c r="C20" s="34" t="s">
+        <v>126</v>
+      </c>
+      <c r="D20" s="34"/>
+      <c r="E20" s="34" t="s">
+        <v>75</v>
+      </c>
+      <c r="F20" s="34" t="s">
+        <v>75</v>
+      </c>
+      <c r="G20" s="34" t="s">
+        <v>127</v>
+      </c>
+      <c r="H20" s="35" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="34" t="s">
+        <v>128</v>
+      </c>
+      <c r="B21" s="34" t="s">
+        <v>27</v>
+      </c>
+      <c r="C21" s="34" t="s">
+        <v>129</v>
+      </c>
+      <c r="D21" s="34"/>
+      <c r="E21" s="34" t="s">
+        <v>130</v>
+      </c>
+      <c r="F21" s="34" t="s">
+        <v>83</v>
+      </c>
+      <c r="G21" s="34" t="s">
+        <v>131</v>
+      </c>
+      <c r="H21" s="35" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="32" t="s">
-        <v>118</v>
-      </c>
-      <c r="B18" s="32" t="s">
-        <v>25</v>
-      </c>
-      <c r="C18" s="32" t="s">
-        <v>119</v>
-      </c>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32" t="s">
-        <v>102</v>
-      </c>
-      <c r="F18" s="32" t="s">
-        <v>102</v>
-      </c>
-      <c r="G18" s="32" t="s">
-        <v>120</v>
-      </c>
-      <c r="H18" s="33" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="32" t="s">
-        <v>121</v>
-      </c>
-      <c r="B19" s="32" t="s">
-        <v>25</v>
-      </c>
-      <c r="C19" s="32" t="s">
-        <v>122</v>
-      </c>
-      <c r="D19" s="32"/>
-      <c r="E19" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="F19" s="32" t="s">
-        <v>69</v>
-      </c>
-      <c r="G19" s="32" t="s">
-        <v>123</v>
-      </c>
-      <c r="H19" s="33" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="32" t="s">
-        <v>124</v>
-      </c>
-      <c r="B20" s="32" t="s">
-        <v>25</v>
-      </c>
-      <c r="C20" s="32" t="s">
-        <v>125</v>
-      </c>
-      <c r="D20" s="32"/>
-      <c r="E20" s="32" t="s">
-        <v>74</v>
-      </c>
-      <c r="F20" s="32" t="s">
-        <v>74</v>
-      </c>
-      <c r="G20" s="32" t="s">
-        <v>126</v>
-      </c>
-      <c r="H20" s="33" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="32" t="s">
-        <v>127</v>
-      </c>
-      <c r="B21" s="32" t="s">
-        <v>26</v>
-      </c>
-      <c r="C21" s="32" t="s">
-        <v>128</v>
-      </c>
-      <c r="D21" s="32"/>
-      <c r="E21" s="32" t="s">
-        <v>129</v>
-      </c>
-      <c r="F21" s="32" t="s">
-        <v>82</v>
-      </c>
-      <c r="G21" s="32" t="s">
-        <v>130</v>
-      </c>
-      <c r="H21" s="33" t="s">
-        <v>11</v>
-      </c>
-    </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="19" t="s">
-        <v>131</v>
+      <c r="A23" s="20" t="s">
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -3663,11 +3723,11 @@
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
+    <oddHeader>&amp;C&amp;10 Multimédia Glory Guinée SARLU</oddHeader>
+    <oddFooter>&amp;C&amp;9 Page &amp;P sur &amp;N</oddFooter>
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -3687,247 +3747,247 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>132</v>
+      <c r="A1" s="2" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>133</v>
+      <c r="A2" s="21" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="B4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>136</v>
       </c>
+      <c r="C4" s="6" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="32" t="s">
+      <c r="A5" s="34" t="s">
+        <v>69</v>
+      </c>
+      <c r="B5" s="36" t="s">
         <v>68</v>
       </c>
-      <c r="B5" s="34" t="s">
-        <v>67</v>
-      </c>
-      <c r="C5" s="32" t="str">
+      <c r="C5" s="34" t="str">
         <f aca="false">IF(B5="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B5,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Gestion administrative</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="B6" s="36" t="s">
         <v>77</v>
       </c>
-      <c r="B6" s="34" t="s">
-        <v>76</v>
-      </c>
-      <c r="C6" s="32" t="str">
+      <c r="C6" s="34" t="str">
         <f aca="false">IF(B6="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B6,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Conventions, avenants et contrats</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="B7" s="36" t="s">
         <v>80</v>
       </c>
-      <c r="B7" s="34" t="s">
-        <v>79</v>
-      </c>
-      <c r="C7" s="32" t="str">
+      <c r="C7" s="34" t="str">
         <f aca="false">IF(B7="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B7,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Conventions, avenants et contrats</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="32" t="s">
+      <c r="A8" s="34" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8" s="36" t="s">
         <v>89</v>
       </c>
-      <c r="B8" s="34" t="s">
-        <v>88</v>
-      </c>
-      <c r="C8" s="32" t="str">
+      <c r="C8" s="34" t="str">
         <f aca="false">IF(B8="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B8,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Relations avec les partenaires</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="35" t="s">
-        <v>137</v>
-      </c>
-      <c r="B9" s="34" t="s">
-        <v>91</v>
-      </c>
-      <c r="C9" s="32" t="str">
+      <c r="A9" s="37" t="s">
+        <v>138</v>
+      </c>
+      <c r="B9" s="36" t="s">
+        <v>92</v>
+      </c>
+      <c r="C9" s="34" t="str">
         <f aca="false">IF(B9="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B9,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Relations avec les partenaires</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="32" t="s">
+      <c r="A10" s="34" t="s">
+        <v>86</v>
+      </c>
+      <c r="B10" s="36" t="s">
         <v>85</v>
       </c>
-      <c r="B10" s="34" t="s">
-        <v>84</v>
-      </c>
-      <c r="C10" s="32" t="str">
+      <c r="C10" s="34" t="str">
         <f aca="false">IF(B10="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B10,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Conventions, avenants et contrats</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="35" t="s">
+      <c r="A11" s="37" t="s">
+        <v>98</v>
+      </c>
+      <c r="B11" s="36" t="s">
         <v>97</v>
       </c>
-      <c r="B11" s="34" t="s">
-        <v>96</v>
-      </c>
-      <c r="C11" s="32" t="str">
+      <c r="C11" s="34" t="str">
         <f aca="false">IF(B11="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B11,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Relations avec les partenaires</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="35" t="s">
+      <c r="A12" s="37" t="s">
+        <v>102</v>
+      </c>
+      <c r="B12" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="34" t="s">
-        <v>100</v>
-      </c>
-      <c r="C12" s="32" t="str">
+      <c r="C12" s="34" t="str">
         <f aca="false">IF(B12="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B12,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Contrôle et suivi financier</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="32" t="s">
-        <v>138</v>
-      </c>
-      <c r="B13" s="34" t="s">
-        <v>104</v>
-      </c>
-      <c r="C13" s="32" t="str">
+      <c r="A13" s="34" t="s">
+        <v>139</v>
+      </c>
+      <c r="B13" s="36" t="s">
+        <v>105</v>
+      </c>
+      <c r="C13" s="34" t="str">
         <f aca="false">IF(B13="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B13,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Contrôle et suivi financier</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="32" t="s">
+      <c r="A14" s="34" t="s">
+        <v>110</v>
+      </c>
+      <c r="B14" s="36" t="s">
         <v>109</v>
       </c>
-      <c r="B14" s="34" t="s">
-        <v>108</v>
-      </c>
-      <c r="C14" s="32" t="str">
+      <c r="C14" s="34" t="str">
         <f aca="false">IF(B14="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B14,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Contrôle et suivi financier</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="35" t="s">
-        <v>139</v>
-      </c>
-      <c r="B15" s="34" t="s">
-        <v>111</v>
-      </c>
-      <c r="C15" s="32" t="str">
+      <c r="A15" s="37" t="s">
+        <v>140</v>
+      </c>
+      <c r="B15" s="36" t="s">
+        <v>112</v>
+      </c>
+      <c r="C15" s="34" t="str">
         <f aca="false">IF(B15="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B15,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Contrôle et suivi financier</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="32" t="s">
+      <c r="A16" s="34" t="s">
+        <v>117</v>
+      </c>
+      <c r="B16" s="36" t="s">
         <v>116</v>
       </c>
-      <c r="B16" s="34" t="s">
-        <v>115</v>
-      </c>
-      <c r="C16" s="32" t="str">
+      <c r="C16" s="34" t="str">
         <f aca="false">IF(B16="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B16,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Contrôle et suivi financier</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="35" t="s">
+      <c r="A17" s="37" t="s">
+        <v>120</v>
+      </c>
+      <c r="B17" s="36" t="s">
         <v>119</v>
       </c>
-      <c r="B17" s="34" t="s">
-        <v>118</v>
-      </c>
-      <c r="C17" s="32" t="str">
+      <c r="C17" s="34" t="str">
         <f aca="false">IF(B17="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B17,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Pilotage de l’équipe</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="35" t="s">
+      <c r="A18" s="37" t="s">
+        <v>123</v>
+      </c>
+      <c r="B18" s="36" t="s">
         <v>122</v>
       </c>
-      <c r="B18" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="C18" s="32" t="str">
+      <c r="C18" s="34" t="str">
         <f aca="false">IF(B18="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B18,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Pilotage de l’équipe</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="35" t="s">
+      <c r="A19" s="37" t="s">
+        <v>126</v>
+      </c>
+      <c r="B19" s="36" t="s">
         <v>125</v>
       </c>
-      <c r="B19" s="34" t="s">
-        <v>124</v>
-      </c>
-      <c r="C19" s="32" t="str">
+      <c r="C19" s="34" t="str">
         <f aca="false">IF(B19="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B19,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Pilotage de l’équipe</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="32" t="s">
-        <v>140</v>
-      </c>
-      <c r="B20" s="34"/>
-      <c r="C20" s="32" t="str">
+      <c r="A20" s="34" t="s">
+        <v>141</v>
+      </c>
+      <c r="B20" s="36"/>
+      <c r="C20" s="34" t="str">
         <f aca="false">IF(B20="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B20,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Rôle du poste</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="32" t="s">
-        <v>141</v>
-      </c>
-      <c r="B21" s="34" t="s">
-        <v>71</v>
-      </c>
-      <c r="C21" s="32" t="str">
+      <c r="A21" s="34" t="s">
+        <v>142</v>
+      </c>
+      <c r="B21" s="36" t="s">
+        <v>72</v>
+      </c>
+      <c r="C21" s="34" t="str">
         <f aca="false">IF(B21="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B21,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Gestion administrative</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="32" t="s">
-        <v>142</v>
-      </c>
-      <c r="B22" s="34" t="s">
-        <v>127</v>
-      </c>
-      <c r="C22" s="32" t="str">
+      <c r="A22" s="34" t="s">
+        <v>143</v>
+      </c>
+      <c r="B22" s="36" t="s">
+        <v>128</v>
+      </c>
+      <c r="C22" s="34" t="str">
         <f aca="false">IF(B22="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B22,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Demandes de la Direction</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
+    <oddHeader>&amp;C&amp;10 Multimédia Glory Guinée SARLU</oddHeader>
+    <oddFooter>&amp;C&amp;9 Page &amp;P sur &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Explique chaque terme de référence : page web, Excel et logo pour la fiche
Onglet Termes de référence de la page : clic sur chaque ligne pour lire
En simple / Concrètement / C'est bien fait quand, avec lexique et points à
clarifier. Feuille Excel équivalente. Logo sur fond blanc pour la fiche.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Frq6RJqehZfzo9cs9xsRRC
</commit_message>
<xml_diff>
--- a/tableau-de-bord-responsable-administratif/tableau-de-bord-responsable-administratif.xlsx
+++ b/tableau-de-bord-responsable-administratif/tableau-de-bord-responsable-administratif.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="228">
   <si>
     <t xml:space="preserve">Multimédia Glory Guinée SARLU</t>
   </si>
@@ -427,13 +427,16 @@
     <t xml:space="preserve">Une mission récurrente n’est jamais « terminée » : « Fait » veut dire fait pour la période en cours. À chaque nouvelle période, remettez la colonne H sur « À faire ».</t>
   </si>
   <si>
-    <t xml:space="preserve">Multimédia Glory Guinée SARLU — Termes de référence — Responsable administratif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Texte du document d’origine (orthographe corrigée). Les colonnes B et C indiquent où chaque ligne est suivie dans le classeur.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fonctions</t>
+    <t xml:space="preserve">Multimédia Glory Guinée SARLU — Termes de référence expliqués — Responsable administratif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Texte du document d’origine (orthographe corrigée), puis explication simple de chaque ligne. La colonne C indique où la ligne est suivie dans le classeur.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quand le texte dit « assurer », « veiller » ou « piloter », le responsable répond du résultat, même s’il ne fait pas tout lui-même. Quand il dit « saisir », « classer » ou « enregistrer », c’est une tâche qu’il fait lui-même.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fonction (texte du document)</t>
   </si>
   <si>
     <t xml:space="preserve">Mission suivie (ID)</t>
@@ -442,22 +445,300 @@
     <t xml:space="preserve">Domaine suivi</t>
   </si>
   <si>
+    <t xml:space="preserve">En simple</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concrètement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C’est bien fait quand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À savoir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faire en sorte que l’administration fonctionne bien au quotidien : à jour, organisée, sans retard.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Fixer des règles claires : qui fait quoi, où ranger, quels délais.
+• Repérer ce qui traîne et le corriger.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Il y a peu de retards et on retrouve vite n’importe quel dossier.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S’assurer qu’aucun accord n’est perdu, oublié ou expiré sans que personne ne s’en aperçoive.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Tenir la liste de tous les accords : partenaire, dates de début et de fin, montant.
+• Prévenir la direction avant chaque échéance.
+• Préparer les renouvellements et les avenants.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aucun document n’arrive à échéance sans qu’une décision ait été prise.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lexique : Convention : accord écrit avec un partenaire. Contrat : accord qui engage l’entreprise. Avenant : document qui modifie un accord existant.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Garder une trace officielle et en sécurité de chaque accord.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Enregistrer : noter l’accord dans un registre (numéro, date, partenaire).
+• Conserver : archiver la version signée, en papier et en scan, bien rangée et sauvegardée.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">On retrouve un contrat signé en quelques minutes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Être l’interlocuteur administratif des partenaires, pas celui qui négocie les accords.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Répondre à leurs demandes et leur envoyer les documents.
+• Relancer quand il manque quelque chose.
+• Garder une trace des échanges.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aucune demande de partenaire ne reste sans réponse.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Recenser les documents à transmettre (protocole, émargements, conventions, …)</t>
   </si>
   <si>
+    <t xml:space="preserve">Faire la liste de tout ce qu’il faut envoyer à chaque partenaire, et vérifier qu’on l’a bien.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Comparer ce qui est attendu avec ce qui est reçu.
+• Relancer les documents manquants.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La liste est complète et rien n’est oublié au moment d’envoyer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lexique : Protocole : document qui fixe les règles de collaboration. Émargements : feuilles de présence signées par les personnes présentes à une séance, une formation ou une activité.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Copier les informations clés de chaque convention dans le fichier ou le logiciel de suivi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Noter les dates, les montants et ce que chaque partie doit fournir.
+• C’est ce qui permet de savoir à tout moment où en est chaque convention.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toutes les conventions sont dans l’outil de suivi, avec des informations exactes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À ne pas confondre : Différence avec « Enregistrer et conserver » : l’enregistrement sert à archiver, la saisie sert à suivre.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C’est la dernière vérification avant de transmettre un dossier.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Vérifier que tout est présent, signé et lisible.
+• Vérifier que les noms, les dates et les montants sont justes.
+• Une pièce manquante peut bloquer un paiement ou retarder un dossier.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les dossiers sont acceptés du premier coup, sans demande de complément.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relire les documents pour s’assurer qu’ils sont corrects et conformes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Vérifier les signatures, les dates et les mentions obligatoires.
+• Vérifier que les documents ne se contredisent pas entre eux.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peu d’erreurs passent entre les mailles.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Vérifier la saisie mensuelle (anomalie, cohérence des plannings)</t>
   </si>
   <si>
+    <t xml:space="preserve">Chaque mois, relire ce qui a été saisi pour repérer les erreurs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Une anomalie est une erreur, un doublon, un oubli ou un montant qui paraît étrange.
+• La cohérence des plannings veut dire que les horaires, les présences et les affectations correspondent à la réalité : une personne ne peut pas être à deux endroits à la fois.
+• Cette saisie sert souvent à payer ou à facturer, d’où l’importance de la vérifier.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les anomalies sont trouvées et corrigées avant la clôture du mois.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ranger les preuves : factures, reçus, feuilles de présence, bons de commande.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Adopter une méthode simple (par mois, par partenaire ou par type) et s’y tenir.
+• Cela permet de justifier un chiffre en cas de question ou de contrôle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chaque chiffre important a sa preuve, facile à retrouver.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Établir les tableaux de bord mensuels en lien avec le cadre intermédiaire financier</t>
   </si>
   <si>
+    <t xml:space="preserve">Produire chaque mois une synthèse chiffrée de l’activité administrative. C’est ce que permet le tableau de bord du responsable administratif.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Récupérer les chiffres auprès du responsable financier.
+• Les mettre en forme et les comparer aux objectifs.
+• Les présenter à la direction.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le tableau est prêt à date fixe et la direction s’en sert pour décider.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À confirmer : « Cadre intermédiaire financier » désigne probablement le responsable financier de niveau intermédiaire. À confirmer avec le Directeur Général.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suivre les paiements.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Vérifier ce qui a été payé et ce qui ne l’est pas encore.
+• Repérer les retards, relancer ou alerter la direction.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aucun retard de paiement ne passe inaperçu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À confirmer : À préciser : cela concerne-t-il les paiements reçus des partenaires, ceux que l’entreprise doit payer, ou les deux ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diriger l’équipe.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Fixer les objectifs et les priorités.
+• Répartir le travail.
+• Faire un point régulier et suivre les résultats.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L’équipe sait ce qu’on attend d’elle et atteint ses objectifs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S’assurer que l’équipe peut travailler dans de bonnes conditions.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Donner les outils et les consignes.
+• Résoudre les blocages.
+• Prévoir un remplacement en cas d’absence.
+• Garder une bonne ambiance de travail.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peu de blocages restent ouverts et le travail continue même en cas d’absence.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faire en sorte que chacun sache quoi faire, et quand.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Transmettre les demandes de la direction.
+• Éviter qu’une tâche soit faite deux fois ou oubliée.
+• Faire circuler l’information.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les tâches s’enchaînent sans doublon ni oubli.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Chargé de la gestion administrative</t>
   </si>
   <si>
+    <t xml:space="preserve">C’est l’intitulé du rôle : cette personne tient l’administration de l’entreprise en ordre.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Les dossiers, les courriers, les contrats et les rendez-vous passent par elle, ou sous son contrôle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personne ne cherche un document et aucune échéance n’est ratée.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Effectue le traitement administratif de dossiers (prise de rendez-vous, rédaction du courrier, classement des dossiers, saisie de documents ou du budget).</t>
   </si>
   <si>
+    <t xml:space="preserve">C’est le travail courant, avec cinq tâches précises.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Prendre les rendez-vous et tenir l’agenda.
+• Rédiger les courriers et les réponses officielles.
+• Classer les dossiers, en papier et en numérique.
+• Saisir les documents dans les fichiers de l’entreprise.
+• Saisir le budget : entrer les montants prévus et dépensés.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le courrier part à temps et le budget est à jour.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Accomplir toutes autres tâches qui lui seront confiées par le Directeur Général</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C’est une clause ouverte : le Directeur Général peut ajouter des tâches liées au poste.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Noter chaque demande : date, contenu, échéance.
+• Cela évite les oublis et permet de montrer ce qui a été fait.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les demandes sont traitées dans les délais.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conseil : Pour une tâche importante ou inhabituelle, demandez une confirmation écrite. Cette clause couvre normalement des tâches cohérentes avec le poste ; les limites exactes dépendent du contrat de travail.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PETIT LEXIQUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Convention</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accord écrit avec un partenaire : qui fait quoi, pendant combien de temps, à quelles conditions.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contrat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accord qui engage l’entreprise, avec un client, un fournisseur ou un salarié.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avenant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Document qui modifie un accord existant (durée, montant, date) sans tout refaire.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protocole</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Document qui fixe les règles de collaboration avec un partenaire.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Émargement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feuille de présence signée par les personnes présentes à une séance, une formation ou une activité.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Justificatif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preuve d’une dépense ou d’une activité : facture, reçu, bon de commande, feuille de présence.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anomalie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Erreur, doublon, oubli ou montant qui paraît étrange dans une saisie.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">À CLARIFIER AVEC LE DIRECTEUR GÉNÉRAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Qui est exactement le « cadre intermédiaire financier » (ligne « Établir les tableaux de bord mensuels ») ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Que recouvre « règlements » (ligne « Suivre les règlements ») : les encaissements, les paiements, ou les deux ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Quelles sont les limites de la dernière clause (« toutes autres tâches confiées par le Directeur Général ») ?</t>
   </si>
 </sst>
 </file>
@@ -704,7 +985,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="41">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -849,12 +1130,24 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="3" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1552,11 +1845,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="83873311"/>
-        <c:axId val="29672029"/>
+        <c:axId val="74589961"/>
+        <c:axId val="11667807"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="83873311"/>
+        <c:axId val="74589961"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1588,7 +1881,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29672029"/>
+        <c:crossAx val="11667807"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1596,7 +1889,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="29672029"/>
+        <c:axId val="11667807"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1628,7 +1921,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83873311"/>
+        <c:crossAx val="74589961"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1954,11 +2247,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="65983716"/>
-        <c:axId val="35577680"/>
+        <c:axId val="48134109"/>
+        <c:axId val="96045634"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="65983716"/>
+        <c:axId val="48134109"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1990,7 +2283,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="35577680"/>
+        <c:crossAx val="96045634"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1998,7 +2291,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="35577680"/>
+        <c:axId val="96045634"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2030,7 +2323,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65983716"/>
+        <c:crossAx val="48134109"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3738,12 +4031,16 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="92"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="56"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3756,229 +4053,531 @@
         <v>134</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="20" t="s">
         <v>135</v>
       </c>
-      <c r="B4" s="6" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="B5" s="6" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="34" t="s">
+      <c r="C5" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="36" t="s">
         <v>69</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B6" s="37" t="s">
         <v>68</v>
-      </c>
-      <c r="C5" s="34" t="str">
-        <f aca="false">IF(B5="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B5,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
-        <v>Gestion administrative</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="34" t="s">
-        <v>78</v>
-      </c>
-      <c r="B6" s="36" t="s">
-        <v>77</v>
       </c>
       <c r="C6" s="34" t="str">
         <f aca="false">IF(B6="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B6,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
-        <v>Conventions, avenants et contrats</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="37" t="s">
-        <v>81</v>
-      </c>
-      <c r="B7" s="36" t="s">
-        <v>80</v>
+        <v>Gestion administrative</v>
+      </c>
+      <c r="D6" s="34" t="s">
+        <v>143</v>
+      </c>
+      <c r="E6" s="34" t="s">
+        <v>144</v>
+      </c>
+      <c r="F6" s="34" t="s">
+        <v>145</v>
+      </c>
+      <c r="G6" s="34"/>
+    </row>
+    <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" s="37" t="s">
+        <v>77</v>
       </c>
       <c r="C7" s="34" t="str">
         <f aca="false">IF(B7="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B7,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Conventions, avenants et contrats</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="34" t="s">
-        <v>90</v>
-      </c>
-      <c r="B8" s="36" t="s">
-        <v>89</v>
+      <c r="D7" s="34" t="s">
+        <v>146</v>
+      </c>
+      <c r="E7" s="34" t="s">
+        <v>147</v>
+      </c>
+      <c r="F7" s="34" t="s">
+        <v>148</v>
+      </c>
+      <c r="G7" s="34" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="38" t="s">
+        <v>81</v>
+      </c>
+      <c r="B8" s="37" t="s">
+        <v>80</v>
       </c>
       <c r="C8" s="34" t="str">
         <f aca="false">IF(B8="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B8,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
-        <v>Relations avec les partenaires</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="37" t="s">
-        <v>138</v>
-      </c>
-      <c r="B9" s="36" t="s">
-        <v>92</v>
+        <v>Conventions, avenants et contrats</v>
+      </c>
+      <c r="D8" s="34" t="s">
+        <v>150</v>
+      </c>
+      <c r="E8" s="34" t="s">
+        <v>151</v>
+      </c>
+      <c r="F8" s="34" t="s">
+        <v>152</v>
+      </c>
+      <c r="G8" s="34"/>
+    </row>
+    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="36" t="s">
+        <v>90</v>
+      </c>
+      <c r="B9" s="37" t="s">
+        <v>89</v>
       </c>
       <c r="C9" s="34" t="str">
         <f aca="false">IF(B9="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B9,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Relations avec les partenaires</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="34" t="s">
-        <v>86</v>
-      </c>
-      <c r="B10" s="36" t="s">
-        <v>85</v>
+      <c r="D9" s="34" t="s">
+        <v>153</v>
+      </c>
+      <c r="E9" s="34" t="s">
+        <v>154</v>
+      </c>
+      <c r="F9" s="34" t="s">
+        <v>155</v>
+      </c>
+      <c r="G9" s="34"/>
+    </row>
+    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="38" t="s">
+        <v>156</v>
+      </c>
+      <c r="B10" s="37" t="s">
+        <v>92</v>
       </c>
       <c r="C10" s="34" t="str">
         <f aca="false">IF(B10="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B10,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
-        <v>Conventions, avenants et contrats</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="37" t="s">
-        <v>98</v>
-      </c>
-      <c r="B11" s="36" t="s">
-        <v>97</v>
+        <v>Relations avec les partenaires</v>
+      </c>
+      <c r="D10" s="34" t="s">
+        <v>157</v>
+      </c>
+      <c r="E10" s="34" t="s">
+        <v>158</v>
+      </c>
+      <c r="F10" s="34" t="s">
+        <v>159</v>
+      </c>
+      <c r="G10" s="34" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="36" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11" s="37" t="s">
+        <v>85</v>
       </c>
       <c r="C11" s="34" t="str">
         <f aca="false">IF(B11="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B11,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
-        <v>Relations avec les partenaires</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="37" t="s">
-        <v>102</v>
-      </c>
-      <c r="B12" s="36" t="s">
-        <v>101</v>
+        <v>Conventions, avenants et contrats</v>
+      </c>
+      <c r="D11" s="34" t="s">
+        <v>161</v>
+      </c>
+      <c r="E11" s="34" t="s">
+        <v>162</v>
+      </c>
+      <c r="F11" s="34" t="s">
+        <v>163</v>
+      </c>
+      <c r="G11" s="34" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="38" t="s">
+        <v>98</v>
+      </c>
+      <c r="B12" s="37" t="s">
+        <v>97</v>
       </c>
       <c r="C12" s="34" t="str">
         <f aca="false">IF(B12="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B12,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
-        <v>Contrôle et suivi financier</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="34" t="s">
-        <v>139</v>
-      </c>
-      <c r="B13" s="36" t="s">
-        <v>105</v>
+        <v>Relations avec les partenaires</v>
+      </c>
+      <c r="D12" s="34" t="s">
+        <v>165</v>
+      </c>
+      <c r="E12" s="34" t="s">
+        <v>166</v>
+      </c>
+      <c r="F12" s="34" t="s">
+        <v>167</v>
+      </c>
+      <c r="G12" s="34"/>
+    </row>
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="38" t="s">
+        <v>102</v>
+      </c>
+      <c r="B13" s="37" t="s">
+        <v>101</v>
       </c>
       <c r="C13" s="34" t="str">
         <f aca="false">IF(B13="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B13,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Contrôle et suivi financier</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="34" t="s">
-        <v>110</v>
-      </c>
-      <c r="B14" s="36" t="s">
-        <v>109</v>
+      <c r="D13" s="34" t="s">
+        <v>168</v>
+      </c>
+      <c r="E13" s="34" t="s">
+        <v>169</v>
+      </c>
+      <c r="F13" s="34" t="s">
+        <v>170</v>
+      </c>
+      <c r="G13" s="34"/>
+    </row>
+    <row r="14" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="36" t="s">
+        <v>171</v>
+      </c>
+      <c r="B14" s="37" t="s">
+        <v>105</v>
       </c>
       <c r="C14" s="34" t="str">
         <f aca="false">IF(B14="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B14,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Contrôle et suivi financier</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="37" t="s">
-        <v>140</v>
-      </c>
-      <c r="B15" s="36" t="s">
-        <v>112</v>
+      <c r="D14" s="34" t="s">
+        <v>172</v>
+      </c>
+      <c r="E14" s="34" t="s">
+        <v>173</v>
+      </c>
+      <c r="F14" s="34" t="s">
+        <v>174</v>
+      </c>
+      <c r="G14" s="34"/>
+    </row>
+    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="36" t="s">
+        <v>110</v>
+      </c>
+      <c r="B15" s="37" t="s">
+        <v>109</v>
       </c>
       <c r="C15" s="34" t="str">
         <f aca="false">IF(B15="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B15,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Contrôle et suivi financier</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="34" t="s">
-        <v>117</v>
-      </c>
-      <c r="B16" s="36" t="s">
-        <v>116</v>
+      <c r="D15" s="34" t="s">
+        <v>175</v>
+      </c>
+      <c r="E15" s="34" t="s">
+        <v>176</v>
+      </c>
+      <c r="F15" s="34" t="s">
+        <v>177</v>
+      </c>
+      <c r="G15" s="34"/>
+    </row>
+    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="38" t="s">
+        <v>178</v>
+      </c>
+      <c r="B16" s="37" t="s">
+        <v>112</v>
       </c>
       <c r="C16" s="34" t="str">
         <f aca="false">IF(B16="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B16,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Contrôle et suivi financier</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="37" t="s">
-        <v>120</v>
-      </c>
-      <c r="B17" s="36" t="s">
-        <v>119</v>
+      <c r="D16" s="34" t="s">
+        <v>179</v>
+      </c>
+      <c r="E16" s="34" t="s">
+        <v>180</v>
+      </c>
+      <c r="F16" s="34" t="s">
+        <v>181</v>
+      </c>
+      <c r="G16" s="34" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="36" t="s">
+        <v>117</v>
+      </c>
+      <c r="B17" s="37" t="s">
+        <v>116</v>
       </c>
       <c r="C17" s="34" t="str">
         <f aca="false">IF(B17="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B17,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
-        <v>Pilotage de l’équipe</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="37" t="s">
-        <v>123</v>
-      </c>
-      <c r="B18" s="36" t="s">
-        <v>122</v>
+        <v>Contrôle et suivi financier</v>
+      </c>
+      <c r="D17" s="34" t="s">
+        <v>183</v>
+      </c>
+      <c r="E17" s="34" t="s">
+        <v>184</v>
+      </c>
+      <c r="F17" s="34" t="s">
+        <v>185</v>
+      </c>
+      <c r="G17" s="34" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="B18" s="37" t="s">
+        <v>119</v>
       </c>
       <c r="C18" s="34" t="str">
         <f aca="false">IF(B18="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B18,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Pilotage de l’équipe</v>
       </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="37" t="s">
-        <v>126</v>
-      </c>
-      <c r="B19" s="36" t="s">
-        <v>125</v>
+      <c r="D18" s="34" t="s">
+        <v>187</v>
+      </c>
+      <c r="E18" s="34" t="s">
+        <v>188</v>
+      </c>
+      <c r="F18" s="34" t="s">
+        <v>189</v>
+      </c>
+      <c r="G18" s="34"/>
+    </row>
+    <row r="19" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="38" t="s">
+        <v>123</v>
+      </c>
+      <c r="B19" s="37" t="s">
+        <v>122</v>
       </c>
       <c r="C19" s="34" t="str">
         <f aca="false">IF(B19="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B19,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Pilotage de l’équipe</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="34" t="s">
-        <v>141</v>
-      </c>
-      <c r="B20" s="36"/>
+      <c r="D19" s="34" t="s">
+        <v>190</v>
+      </c>
+      <c r="E19" s="34" t="s">
+        <v>191</v>
+      </c>
+      <c r="F19" s="34" t="s">
+        <v>192</v>
+      </c>
+      <c r="G19" s="34"/>
+    </row>
+    <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="38" t="s">
+        <v>126</v>
+      </c>
+      <c r="B20" s="37" t="s">
+        <v>125</v>
+      </c>
       <c r="C20" s="34" t="str">
         <f aca="false">IF(B20="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B20,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
-        <v>Rôle du poste</v>
-      </c>
+        <v>Pilotage de l’équipe</v>
+      </c>
+      <c r="D20" s="34" t="s">
+        <v>193</v>
+      </c>
+      <c r="E20" s="34" t="s">
+        <v>194</v>
+      </c>
+      <c r="F20" s="34" t="s">
+        <v>195</v>
+      </c>
+      <c r="G20" s="34"/>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="34" t="s">
-        <v>142</v>
-      </c>
-      <c r="B21" s="36" t="s">
-        <v>72</v>
-      </c>
+      <c r="A21" s="36" t="s">
+        <v>196</v>
+      </c>
+      <c r="B21" s="37"/>
       <c r="C21" s="34" t="str">
         <f aca="false">IF(B21="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B21,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
-        <v>Gestion administrative</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="34" t="s">
-        <v>143</v>
-      </c>
-      <c r="B22" s="36" t="s">
-        <v>128</v>
+        <v>Rôle du poste</v>
+      </c>
+      <c r="D21" s="34" t="s">
+        <v>197</v>
+      </c>
+      <c r="E21" s="34" t="s">
+        <v>198</v>
+      </c>
+      <c r="F21" s="34" t="s">
+        <v>199</v>
+      </c>
+      <c r="G21" s="34"/>
+    </row>
+    <row r="22" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="36" t="s">
+        <v>200</v>
+      </c>
+      <c r="B22" s="37" t="s">
+        <v>72</v>
       </c>
       <c r="C22" s="34" t="str">
         <f aca="false">IF(B22="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B22,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
+        <v>Gestion administrative</v>
+      </c>
+      <c r="D22" s="34" t="s">
+        <v>201</v>
+      </c>
+      <c r="E22" s="34" t="s">
+        <v>202</v>
+      </c>
+      <c r="F22" s="34" t="s">
+        <v>203</v>
+      </c>
+      <c r="G22" s="34"/>
+    </row>
+    <row r="23" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="36" t="s">
+        <v>204</v>
+      </c>
+      <c r="B23" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="C23" s="34" t="str">
+        <f aca="false">IF(B23="","Rôle du poste",IFERROR(INDEX(Missions!$B$5:$B$21,MATCH(B23,Missions!$A$5:$A$21,0)),"ID inconnu"))</f>
         <v>Demandes de la Direction</v>
+      </c>
+      <c r="D23" s="34" t="s">
+        <v>205</v>
+      </c>
+      <c r="E23" s="34" t="s">
+        <v>206</v>
+      </c>
+      <c r="F23" s="34" t="s">
+        <v>207</v>
+      </c>
+      <c r="G23" s="34" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="B25" s="5"/>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="B26" s="39" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="22" t="s">
+        <v>212</v>
+      </c>
+      <c r="B27" s="39" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="22" t="s">
+        <v>214</v>
+      </c>
+      <c r="B28" s="39" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="22" t="s">
+        <v>216</v>
+      </c>
+      <c r="B29" s="39" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="22" t="s">
+        <v>218</v>
+      </c>
+      <c r="B30" s="39" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="22" t="s">
+        <v>220</v>
+      </c>
+      <c r="B31" s="39" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="22" t="s">
+        <v>222</v>
+      </c>
+      <c r="B32" s="39" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="B34" s="5"/>
+      <c r="C34" s="5"/>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="40" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="40" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="40" t="s">
+        <v>227</v>
       </c>
     </row>
   </sheetData>

</xml_diff>